<commit_message>
update LAES turbine case
</commit_message>
<xml_diff>
--- a/projects/LAES_turbine/simulation_cases.xlsx
+++ b/projects/LAES_turbine/simulation_cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/roagr_dtu_dk/Documents/Roberto/Projects/barotropy/projects/DTU_2phaseTurbine/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/roagr_dtu_dk/Documents/Roberto/Projects/barotropy/projects/LAES_turbine/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_7FB4EEAC829E42EF5BBCD4D8176F1B64A0B46118" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{268E2637-C79D-495C-8316-128D5F74CB84}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="11_7FB4EEAC829E42EF5BBCD4D8176F1B64A0B46118" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{997508E2-D633-4669-B172-2FDD463C253B}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>index</t>
   </si>
@@ -59,9 +59,6 @@
     <t>nitrogen</t>
   </si>
   <si>
-    <t>multiphase_model</t>
-  </si>
-  <si>
     <t>q_onset</t>
   </si>
   <si>
@@ -72,6 +69,27 @@
   </si>
   <si>
     <t>blending</t>
+  </si>
+  <si>
+    <t>case_equilibrium</t>
+  </si>
+  <si>
+    <t>case_blend_00</t>
+  </si>
+  <si>
+    <t>case_blend_02</t>
+  </si>
+  <si>
+    <t>case_blend_04</t>
+  </si>
+  <si>
+    <t>case_blend_06</t>
+  </si>
+  <si>
+    <t>case_blend_08</t>
+  </si>
+  <si>
+    <t>calculation_type</t>
   </si>
 </sst>
 </file>
@@ -83,7 +101,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,6 +120,12 @@
       <color rgb="FF000000"/>
       <name val="Consolas"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -477,7 +501,7 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.86328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.86328125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="17.73046875" style="2" customWidth="1"/>
     <col min="3" max="3" width="13.1328125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.73046875" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.73046875" style="4" bestFit="1" customWidth="1"/>
@@ -511,20 +535,22 @@
         <v>6</v>
       </c>
       <c r="H1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
@@ -542,7 +568,7 @@
         <v>0.9</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I2" s="8">
         <v>0</v>
@@ -555,7 +581,9 @@
       <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="C3" s="7" t="s">
         <v>7</v>
       </c>
@@ -573,7 +601,7 @@
         <v>0.9</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I3" s="8">
         <v>0</v>
@@ -586,7 +614,9 @@
       <c r="A4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="7"/>
+      <c r="B4" s="7" t="s">
+        <v>14</v>
+      </c>
       <c r="C4" s="7" t="s">
         <v>7</v>
       </c>
@@ -604,7 +634,7 @@
         <v>0.9</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I4" s="8">
         <v>0.02</v>
@@ -617,7 +647,9 @@
       <c r="A5" s="7">
         <v>4</v>
       </c>
-      <c r="B5" s="7"/>
+      <c r="B5" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="C5" s="7" t="s">
         <v>7</v>
       </c>
@@ -635,7 +667,7 @@
         <v>0.9</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I5" s="8">
         <v>0.04</v>
@@ -648,7 +680,9 @@
       <c r="A6" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="7"/>
+      <c r="B6" s="7" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="7" t="s">
         <v>7</v>
       </c>
@@ -666,7 +700,7 @@
         <v>0.9</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I6" s="8">
         <v>0.06</v>
@@ -679,7 +713,9 @@
       <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="7"/>
+      <c r="B7" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="C7" s="7" t="s">
         <v>7</v>
       </c>
@@ -697,7 +733,7 @@
         <v>0.9</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I7" s="8">
         <v>0.08</v>
@@ -707,6 +743,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update projects with latest changes
</commit_message>
<xml_diff>
--- a/projects/LAES_turbine/simulation_cases.xlsx
+++ b/projects/LAES_turbine/simulation_cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/roagr_dtu_dk/Documents/Roberto/Projects/barotropy/projects/LAES_turbine/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_7FB4EEAC829E42EF5BBCD4D8176F1B64A0B46118" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EBE0BB9-E831-42F1-8544-CD5839ABF24F}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="11_7FB4EEAC829E42EF5BBCD4D8176F1B64A0B46118" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30AB429F-F67C-40A8-ACDD-B8DD4BF7577F}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2520" yWindow="2520" windowWidth="14400" windowHeight="8190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>index</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>case_blend_08</t>
+  </si>
+  <si>
+    <t>Simoneau_Hendricks_1</t>
+  </si>
+  <si>
+    <t>Simoneau_Hendricks_2</t>
+  </si>
+  <si>
+    <t>Simoneau_Hendricks_3</t>
   </si>
 </sst>
 </file>
@@ -104,7 +113,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -210,6 +219,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,22 +513,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.1328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.86328125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.1328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.40625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -547,7 +560,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -580,7 +593,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -613,7 +626,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -646,7 +659,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -679,7 +692,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -712,7 +725,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.75">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -742,6 +755,102 @@
         <v>0.08</v>
       </c>
       <c r="J7" s="8">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.75">
+      <c r="A8" s="1">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="3">
+        <v>95</v>
+      </c>
+      <c r="E8" s="4">
+        <v>600000</v>
+      </c>
+      <c r="F8" s="5">
+        <v>250000</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.75">
+      <c r="A9" s="1">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3">
+        <v>94.7</v>
+      </c>
+      <c r="E9" s="4">
+        <v>780000</v>
+      </c>
+      <c r="F9" s="5">
+        <v>210000</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="8">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.75">
+      <c r="A10" s="1">
+        <v>13</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="3">
+        <v>95</v>
+      </c>
+      <c r="E10" s="4">
+        <v>900000</v>
+      </c>
+      <c r="F10" s="5">
+        <v>370000</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0</v>
+      </c>
+      <c r="J10" s="8">
         <v>0.02</v>
       </c>
     </row>

</xml_diff>